<commit_message>
report v3, updated script, moved index.html
</commit_message>
<xml_diff>
--- a/sprint_worklog_report.xlsx
+++ b/sprint_worklog_report.xlsx
@@ -719,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="3">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9.25</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="4">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="5">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="6">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -841,7 +841,82 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.5</v>
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SCRUM Sprint 3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Anton Hedlund</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SCRUM Sprint 3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Calvin Koch</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SCRUM Sprint 3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Einar Eriksson Wahlin</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SCRUM Sprint 3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Klas Widebeck</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SCRUM Sprint 3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Seleman Hassan</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -933,7 +1008,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SCRUM Sprint 2</t>
+          <t>SCRUM Sprint 3</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -954,11 +1029,7 @@
       <c r="I2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -983,7 +1054,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SCRUM Sprint 2</t>
+          <t>SCRUM Sprint 3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1004,11 +1075,7 @@
       <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1033,7 +1100,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SCRUM Sprint 2</t>
+          <t>SCRUM Sprint 3</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1054,11 +1121,7 @@
       <c r="I4" t="n">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1083,7 +1146,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SCRUM Sprint 2</t>
+          <t>SCRUM Sprint 3</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1104,11 +1167,7 @@
       <c r="I5" t="n">
         <v>1</v>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1154,11 +1213,7 @@
       <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1204,11 +1259,7 @@
       <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1254,11 +1305,7 @@
       <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1304,11 +1351,7 @@
       <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1354,11 +1397,7 @@
       <c r="I10" t="n">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1404,11 +1443,7 @@
       <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1454,11 +1489,7 @@
       <c r="I12" t="n">
         <v>1.5</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1504,11 +1535,7 @@
       <c r="I13" t="n">
         <v>1.5</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1554,11 +1581,7 @@
       <c r="I14" t="n">
         <v>1.5</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1606,7 +1629,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>{'type': 'doc', 'version': 1, 'content': [{'type': 'paragraph', 'content': [{'type': 'text', 'text': 'Team Meeting'}], 'attrs': {'localId': 'e10b569c8156'}}]}</t>
+          <t>Team Meeting</t>
         </is>
       </c>
     </row>
@@ -1654,11 +1677,7 @@
       <c r="I16" t="n">
         <v>1.5</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1704,11 +1723,7 @@
       <c r="I17" t="n">
         <v>1.5</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1754,11 +1769,7 @@
       <c r="I18" t="n">
         <v>3</v>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1804,11 +1815,7 @@
       <c r="I19" t="n">
         <v>1</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1854,11 +1861,7 @@
       <c r="I20" t="n">
         <v>0.5</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1904,11 +1907,7 @@
       <c r="I21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2000,11 +1999,7 @@
       <c r="I23" t="n">
         <v>1</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2050,11 +2045,7 @@
       <c r="I24" t="n">
         <v>1</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2100,11 +2091,7 @@
       <c r="I25" t="n">
         <v>1</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2150,11 +2137,7 @@
       <c r="I26" t="n">
         <v>1</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2200,11 +2183,7 @@
       <c r="I27" t="n">
         <v>1</v>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2250,11 +2229,7 @@
       <c r="I28" t="n">
         <v>1</v>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2300,11 +2275,7 @@
       <c r="I29" t="n">
         <v>3</v>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2329,7 +2300,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SCRUM Sprint 1</t>
+          <t>SCRUM Sprint 2</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2350,11 +2321,7 @@
       <c r="I30" t="n">
         <v>1</v>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2400,11 +2367,7 @@
       <c r="I31" t="n">
         <v>3</v>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2450,11 +2413,7 @@
       <c r="I32" t="n">
         <v>0.25</v>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2500,11 +2459,7 @@
       <c r="I33" t="n">
         <v>1</v>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2550,11 +2505,7 @@
       <c r="I34" t="n">
         <v>2</v>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2579,7 +2530,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SCRUM Sprint 2</t>
+          <t>SCRUM Sprint 3</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2600,11 +2551,7 @@
       <c r="I35" t="n">
         <v>2.5</v>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2650,11 +2597,7 @@
       <c r="I36" t="n">
         <v>5</v>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2679,7 +2622,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SCRUM Sprint 2</t>
+          <t>SCRUM Sprint 3</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2700,11 +2643,7 @@
       <c r="I37" t="n">
         <v>5</v>
       </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2750,11 +2689,7 @@
       <c r="I38" t="n">
         <v>0.5</v>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>{'type': 'doc', 'version': 1, 'content': []}</t>
-        </is>
-      </c>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2802,7 +2737,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>{'type': 'doc', 'version': 1, 'content': [{'type': 'paragraph', 'content': [{'type': 'text', 'text': 'The issue has been resolved. '}], 'attrs': {'localId': '250995940946'}}]}</t>
+          <t>The issue has been resolved.</t>
         </is>
       </c>
     </row>
@@ -2873,22 +2808,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-24 00:00:00</t>
+          <t>2026-08-31 00:00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-06 23:59:59</t>
+          <t>2026-09-13 23:59:59</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-08-30 22:00:00</t>
+          <t>2026-08-31 00:00:00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-14 16:33:24</t>
+          <t>2026-09-13 23:59:59</t>
         </is>
       </c>
     </row>
@@ -2918,12 +2853,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-14 16:33:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-28 16:33:24</t>
+          <t>2026-09-27 23:59:59</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2888,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-28 16:33:25</t>
+          <t>2026-09-28 00:00:00</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">

</xml_diff>